<commit_message>
Add Games: - Death Howl - Arc Raiders - Legends of Runeterra - Easy Delivery Co.
</commit_message>
<xml_diff>
--- a/New_Game_Time.xlsx
+++ b/New_Game_Time.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DAVIMUNO\Desktop\GitHub\Game_times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BD9FE4-6D4D-4CFE-B7B5-9A7C57DCE179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BBF7F0-5808-4A13-9B42-C7015C684B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4900" yWindow="4900" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sessions" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="153">
   <si>
     <t>SessionID</t>
   </si>
@@ -430,6 +430,66 @@
   </si>
   <si>
     <t>20/03/26 22:52</t>
+  </si>
+  <si>
+    <t>Death Howl</t>
+  </si>
+  <si>
+    <t>The Outer Zone</t>
+  </si>
+  <si>
+    <t>11 Bit Studios</t>
+  </si>
+  <si>
+    <t>Legends of Runeterra</t>
+  </si>
+  <si>
+    <t>Riot Games</t>
+  </si>
+  <si>
+    <t>Easy Delivery Co.</t>
+  </si>
+  <si>
+    <t>Sam C</t>
+  </si>
+  <si>
+    <t>Oro Interactive</t>
+  </si>
+  <si>
+    <t>ARC Raiders</t>
+  </si>
+  <si>
+    <t>Embark Studios</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/M/MV5BNjA5MTZkOGUtNmQ4Ni00OTI1LWExMDAtOTU1OGI0ZWMzMWM5XkEyXkFqcGc@._V1_FMjpg_UY2048_.jpg</t>
+  </si>
+  <si>
+    <t>Card Game</t>
+  </si>
+  <si>
+    <t>Deckbuilding</t>
+  </si>
+  <si>
+    <t>Turn-Based</t>
+  </si>
+  <si>
+    <t>Cozy</t>
+  </si>
+  <si>
+    <t>Resource Management</t>
+  </si>
+  <si>
+    <t>Time Management</t>
+  </si>
+  <si>
+    <t>Relaxing</t>
+  </si>
+  <si>
+    <t>Third Person Shooter</t>
+  </si>
+  <si>
+    <t>Extraction Gameplay</t>
   </si>
 </sst>
 </file>
@@ -768,17 +828,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F101"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" customWidth="1"/>
-    <col min="5" max="5" width="16.7265625" customWidth="1"/>
-    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -798,7 +858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -818,7 +878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -838,7 +898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -858,7 +918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -878,7 +938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -898,7 +958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -918,7 +978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -938,7 +998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -958,7 +1018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -978,7 +1038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -998,7 +1058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1018,7 +1078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1038,7 +1098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1058,7 +1118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1078,7 +1138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1098,7 +1158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1118,7 +1178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1138,7 +1198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1158,7 +1218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1178,7 +1238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1198,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1218,7 +1278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1238,7 +1298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1258,7 +1318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1278,7 +1338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1298,7 +1358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1318,7 +1378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1338,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1358,7 +1418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1378,7 +1438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1398,7 +1458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1418,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1438,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1458,7 +1518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1478,7 +1538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1498,7 +1558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1518,7 +1578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1538,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1558,7 +1618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1578,7 +1638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1598,7 +1658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1618,7 +1678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1638,7 +1698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1658,7 +1718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1678,7 +1738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1698,7 +1758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1718,7 +1778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1738,7 +1798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1758,7 +1818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1778,7 +1838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1798,7 +1858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1818,7 +1878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1838,7 +1898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1858,7 +1918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1878,7 +1938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1898,7 +1958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1918,7 +1978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1938,7 +1998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1958,7 +2018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1978,7 +2038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1998,7 +2058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2018,7 +2078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2038,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2058,7 +2118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2078,7 +2138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2098,7 +2158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2118,7 +2178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2138,7 +2198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2158,7 +2218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2178,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2198,7 +2258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2218,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2238,7 +2298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2258,7 +2318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2278,7 +2338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2298,7 +2358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2318,7 +2378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2338,7 +2398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2358,7 +2418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2378,7 +2438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2398,7 +2458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2418,7 +2478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2438,7 +2498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2458,7 +2518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2478,7 +2538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2498,7 +2558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2518,7 +2578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2538,7 +2598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2558,7 +2618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2578,7 +2638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2598,7 +2658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2618,7 +2678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2638,7 +2698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2658,7 +2718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2678,7 +2738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2698,7 +2758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2718,7 +2778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2738,7 +2798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2758,7 +2818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2778,7 +2838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2805,16 +2865,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46282368-3B73-4126-9CAF-0F4DBCD18058}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2831,7 +2891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2848,7 +2908,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2865,7 +2925,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2882,7 +2942,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2899,7 +2959,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2916,7 +2976,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2933,7 +2993,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2950,7 +3010,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2967,7 +3027,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2984,7 +3044,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2999,6 +3059,65 @@
       </c>
       <c r="E11" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E15" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3009,9 +3128,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC08066E-E57F-4738-8F85-A08D22304096}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3019,7 +3138,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3027,7 +3146,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3035,7 +3154,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3043,7 +3162,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3051,7 +3170,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3066,14 +3185,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1832BBAE-382C-4D1D-B62A-7A869140B59D}">
-  <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -3081,7 +3200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3089,7 +3208,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3097,7 +3216,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3105,7 +3224,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3113,7 +3232,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3121,7 +3240,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3129,7 +3248,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3137,7 +3256,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3145,7 +3264,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3153,7 +3272,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3161,7 +3280,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3169,7 +3288,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3177,7 +3296,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3185,7 +3304,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3193,7 +3312,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3201,7 +3320,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3209,7 +3328,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3217,7 +3336,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3225,7 +3344,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3233,7 +3352,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3241,7 +3360,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3249,7 +3368,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3257,7 +3376,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3265,7 +3384,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3273,7 +3392,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3281,7 +3400,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3289,12 +3408,20 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3304,10 +3431,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8190EB1-512E-4DA4-9E52-5BE9B6D9B4ED}">
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -3315,7 +3442,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -3323,7 +3450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3331,7 +3458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -3339,7 +3466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -3347,7 +3474,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -3355,7 +3482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -3363,7 +3490,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -3371,7 +3498,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4</v>
       </c>
@@ -3379,7 +3506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -3387,7 +3514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>6</v>
       </c>
@@ -3395,7 +3522,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -3403,7 +3530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
@@ -3411,7 +3538,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7</v>
       </c>
@@ -3419,7 +3546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>8</v>
       </c>
@@ -3427,7 +3554,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>8</v>
       </c>
@@ -3435,7 +3562,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>9</v>
       </c>
@@ -3443,7 +3570,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9</v>
       </c>
@@ -3451,7 +3578,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>10</v>
       </c>
@@ -3459,12 +3586,76 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>10</v>
       </c>
       <c r="B20">
         <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>11</v>
+      </c>
+      <c r="B21">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>12</v>
+      </c>
+      <c r="B23">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>13</v>
+      </c>
+      <c r="B25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>13</v>
+      </c>
+      <c r="B26">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>14</v>
+      </c>
+      <c r="B27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3474,14 +3665,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B10FE8-D90F-4F6D-86B5-00602E8D2AAC}">
-  <dimension ref="A1:B44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -3489,7 +3680,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3497,7 +3688,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3505,7 +3696,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3513,7 +3704,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3521,7 +3712,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3529,7 +3720,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3537,7 +3728,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3545,7 +3736,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3553,7 +3744,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3561,7 +3752,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3569,7 +3760,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3577,7 +3768,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3585,7 +3776,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3593,7 +3784,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3601,7 +3792,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3609,7 +3800,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3617,7 +3808,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3625,7 +3816,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3633,7 +3824,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3641,7 +3832,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3649,7 +3840,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3657,7 +3848,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3665,7 +3856,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3673,7 +3864,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3681,7 +3872,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3689,7 +3880,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3697,7 +3888,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3705,7 +3896,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3713,7 +3904,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3721,7 +3912,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3729,7 +3920,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3737,7 +3928,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3745,7 +3936,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3753,7 +3944,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3761,7 +3952,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3769,7 +3960,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3777,7 +3968,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3785,7 +3976,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3793,7 +3984,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3801,7 +3992,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3809,7 +4000,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3817,7 +4008,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3825,12 +4016,76 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -3840,10 +4095,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95EFE99A-A4A1-483D-95A3-0523528D2F12}">
-  <dimension ref="A1:B55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B79"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -3851,7 +4106,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>4</v>
       </c>
@@ -3859,7 +4114,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>4</v>
       </c>
@@ -3867,7 +4122,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -3875,7 +4130,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3883,7 +4138,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3891,7 +4146,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -3899,7 +4154,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -3907,7 +4162,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -3915,7 +4170,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -3923,7 +4178,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -3931,7 +4186,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -3939,7 +4194,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -3947,7 +4202,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -3955,7 +4210,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -3963,7 +4218,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -3971,7 +4226,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -3979,7 +4234,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -3987,7 +4242,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -3995,7 +4250,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -4003,7 +4258,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -4011,7 +4266,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -4019,7 +4274,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>5</v>
       </c>
@@ -4027,7 +4282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>5</v>
       </c>
@@ -4035,7 +4290,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>5</v>
       </c>
@@ -4043,7 +4298,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>5</v>
       </c>
@@ -4051,7 +4306,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>6</v>
       </c>
@@ -4059,7 +4314,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>6</v>
       </c>
@@ -4067,7 +4322,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>6</v>
       </c>
@@ -4075,7 +4330,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>6</v>
       </c>
@@ -4083,7 +4338,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>6</v>
       </c>
@@ -4091,7 +4346,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>6</v>
       </c>
@@ -4099,7 +4354,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>7</v>
       </c>
@@ -4107,7 +4362,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>7</v>
       </c>
@@ -4115,7 +4370,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>7</v>
       </c>
@@ -4123,7 +4378,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>7</v>
       </c>
@@ -4131,7 +4386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>7</v>
       </c>
@@ -4139,7 +4394,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>7</v>
       </c>
@@ -4147,7 +4402,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>8</v>
       </c>
@@ -4155,7 +4410,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>8</v>
       </c>
@@ -4163,7 +4418,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>8</v>
       </c>
@@ -4171,7 +4426,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>8</v>
       </c>
@@ -4179,7 +4434,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>9</v>
       </c>
@@ -4187,7 +4442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>9</v>
       </c>
@@ -4195,7 +4450,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>9</v>
       </c>
@@ -4203,7 +4458,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -4211,7 +4466,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>9</v>
       </c>
@@ -4219,7 +4474,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>9</v>
       </c>
@@ -4227,7 +4482,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>9</v>
       </c>
@@ -4235,7 +4490,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>10</v>
       </c>
@@ -4243,7 +4498,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>10</v>
       </c>
@@ -4251,7 +4506,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10</v>
       </c>
@@ -4259,7 +4514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10</v>
       </c>
@@ -4267,7 +4522,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10</v>
       </c>
@@ -4275,12 +4530,204 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10</v>
       </c>
       <c r="B55">
         <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>11</v>
+      </c>
+      <c r="B56">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>11</v>
+      </c>
+      <c r="B57">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>11</v>
+      </c>
+      <c r="B58">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>11</v>
+      </c>
+      <c r="B59">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>11</v>
+      </c>
+      <c r="B60">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>11</v>
+      </c>
+      <c r="B61">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>12</v>
+      </c>
+      <c r="B62">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>12</v>
+      </c>
+      <c r="B63">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>12</v>
+      </c>
+      <c r="B64">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>12</v>
+      </c>
+      <c r="B65">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>12</v>
+      </c>
+      <c r="B66">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>12</v>
+      </c>
+      <c r="B67">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>13</v>
+      </c>
+      <c r="B68">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>13</v>
+      </c>
+      <c r="B69">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>13</v>
+      </c>
+      <c r="B70">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>13</v>
+      </c>
+      <c r="B71">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>13</v>
+      </c>
+      <c r="B72">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>13</v>
+      </c>
+      <c r="B73">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>14</v>
+      </c>
+      <c r="B74">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>14</v>
+      </c>
+      <c r="B75">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>14</v>
+      </c>
+      <c r="B76">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>14</v>
+      </c>
+      <c r="B77">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>14</v>
+      </c>
+      <c r="B78">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>14</v>
+      </c>
+      <c r="B79">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sesions: 101- 119
</commit_message>
<xml_diff>
--- a/New_Game_Time.xlsx
+++ b/New_Game_Time.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DAVIMUNO\Desktop\GitHub\Game_times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BBF7F0-5808-4A13-9B42-C7015C684B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1238BF10-F0E8-42C1-9586-0BF4839C91FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -535,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -547,6 +547,8 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -827,18 +829,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F120"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" customWidth="1"/>
+    <col min="5" max="5" width="16.7265625" customWidth="1"/>
+    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +860,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -878,7 +880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -898,7 +900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -918,7 +920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -938,7 +940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -958,7 +960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -978,7 +980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -998,7 +1000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1018,7 +1020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1038,7 +1040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1058,7 +1060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1078,7 +1080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1098,7 +1100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1118,7 +1120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1138,7 +1140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1158,7 +1160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1178,7 +1180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1198,7 +1200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1218,7 +1220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1238,7 +1240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1258,7 +1260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1278,7 +1280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1298,7 +1300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1318,7 +1320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1338,7 +1340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1358,7 +1360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1378,7 +1380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1398,7 +1400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1418,7 +1420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1438,7 +1440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1458,7 +1460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1478,7 +1480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1498,7 +1500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1518,7 +1520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1538,7 +1540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1558,7 +1560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1578,7 +1580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1618,7 +1620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1638,7 +1640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1658,7 +1660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1678,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1698,7 +1700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1718,7 +1720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1738,7 +1740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1758,7 +1760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1778,7 +1780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1798,7 +1800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1818,7 +1820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1838,7 +1840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1858,7 +1860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1878,7 +1880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1898,7 +1900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1918,7 +1920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1938,7 +1940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1958,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1978,7 +1980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1998,7 +2000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2018,7 +2020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2058,7 +2060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2078,7 +2080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2098,7 +2100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2118,7 +2120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2138,7 +2140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2158,7 +2160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2178,7 +2180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2198,7 +2200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2218,7 +2220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2238,7 +2240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2258,7 +2260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2278,7 +2280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2298,7 +2300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2318,7 +2320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2338,7 +2340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2358,7 +2360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2378,7 +2380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2398,7 +2400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2418,7 +2420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2438,7 +2440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2458,7 +2460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2478,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2498,7 +2500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2518,7 +2520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2538,7 +2540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2558,7 +2560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2578,7 +2580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2598,7 +2600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2618,7 +2620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2638,7 +2640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2658,7 +2660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2678,7 +2680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2698,7 +2700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2718,7 +2720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2738,7 +2740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2758,7 +2760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2778,7 +2780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2798,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2818,7 +2820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2838,7 +2840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2856,6 +2858,386 @@
       </c>
       <c r="F101" s="2">
         <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" s="5">
+        <v>46102</v>
+      </c>
+      <c r="D102" s="6">
+        <v>46102.525706018518</v>
+      </c>
+      <c r="E102" s="6">
+        <v>46102.561122685183</v>
+      </c>
+      <c r="F102">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103">
+        <v>7</v>
+      </c>
+      <c r="C103" s="5">
+        <v>46102</v>
+      </c>
+      <c r="D103" s="6">
+        <v>46102.79515046296</v>
+      </c>
+      <c r="E103" s="6">
+        <v>46102.919456018521</v>
+      </c>
+      <c r="F103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104">
+        <v>11</v>
+      </c>
+      <c r="C104" s="5">
+        <v>46103</v>
+      </c>
+      <c r="D104" s="6">
+        <v>46103.619456018518</v>
+      </c>
+      <c r="E104" s="6">
+        <v>46103.636817129627</v>
+      </c>
+      <c r="F104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" s="5">
+        <v>46103</v>
+      </c>
+      <c r="D105" s="6">
+        <v>46103.768761574072</v>
+      </c>
+      <c r="E105" s="6">
+        <v>46103.868761574071</v>
+      </c>
+      <c r="F105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106">
+        <v>10</v>
+      </c>
+      <c r="C106" s="5">
+        <v>46104</v>
+      </c>
+      <c r="D106" s="6">
+        <v>46104.765277777777</v>
+      </c>
+      <c r="E106" s="6">
+        <v>46104.811805555553</v>
+      </c>
+      <c r="F106">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" s="5">
+        <v>46105</v>
+      </c>
+      <c r="D107" s="6">
+        <v>46105.242361111108</v>
+      </c>
+      <c r="E107" s="6">
+        <v>46105.26458333333</v>
+      </c>
+      <c r="F107">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" s="5">
+        <v>46105</v>
+      </c>
+      <c r="D108" s="6">
+        <v>46105.77847222222</v>
+      </c>
+      <c r="E108" s="6">
+        <v>46105.793055555558</v>
+      </c>
+      <c r="F108">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109">
+        <v>10</v>
+      </c>
+      <c r="C109" s="5">
+        <v>46106</v>
+      </c>
+      <c r="D109" s="6">
+        <v>46106.210416666669</v>
+      </c>
+      <c r="E109" s="6">
+        <v>46106.262499999997</v>
+      </c>
+      <c r="F109">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" s="5">
+        <v>46106</v>
+      </c>
+      <c r="D110" s="6">
+        <v>46106.820138888892</v>
+      </c>
+      <c r="E110" s="6">
+        <v>46106.866666666669</v>
+      </c>
+      <c r="F110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111">
+        <v>12</v>
+      </c>
+      <c r="C111" s="5">
+        <v>46107</v>
+      </c>
+      <c r="D111" s="6">
+        <v>46107.723611111112</v>
+      </c>
+      <c r="E111" s="6">
+        <v>46107.753472222219</v>
+      </c>
+      <c r="F111">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112">
+        <v>13</v>
+      </c>
+      <c r="C112" s="5">
+        <v>46108</v>
+      </c>
+      <c r="D112" s="6">
+        <v>46108.767361111109</v>
+      </c>
+      <c r="E112" s="6">
+        <v>46108.897916666669</v>
+      </c>
+      <c r="F112">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113">
+        <v>14</v>
+      </c>
+      <c r="C113" s="5">
+        <v>46109</v>
+      </c>
+      <c r="D113" s="6">
+        <v>46109.333344907405</v>
+      </c>
+      <c r="E113" s="6">
+        <v>46109.355567129627</v>
+      </c>
+      <c r="F113">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>14</v>
+      </c>
+      <c r="C114" s="5">
+        <v>46109</v>
+      </c>
+      <c r="D114" s="6">
+        <v>46109.950011574074</v>
+      </c>
+      <c r="E114" s="6">
+        <v>46110.075706018521</v>
+      </c>
+      <c r="F114">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>14</v>
+      </c>
+      <c r="C115" s="5">
+        <v>46110</v>
+      </c>
+      <c r="D115" s="6">
+        <v>46110.427789351852</v>
+      </c>
+      <c r="E115" s="6">
+        <v>46110.602094907408</v>
+      </c>
+      <c r="F115">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>14</v>
+      </c>
+      <c r="C116" s="5">
+        <v>46110</v>
+      </c>
+      <c r="D116" s="6">
+        <v>46110.81181712963</v>
+      </c>
+      <c r="E116" s="6">
+        <v>46110.873622685183</v>
+      </c>
+      <c r="F116">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>14</v>
+      </c>
+      <c r="C117" s="5">
+        <v>46110</v>
+      </c>
+      <c r="D117" s="6">
+        <v>46110.887511574074</v>
+      </c>
+      <c r="E117" s="6">
+        <v>46110.956956018519</v>
+      </c>
+      <c r="F117">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>2</v>
+      </c>
+      <c r="C118" s="5">
+        <v>46110</v>
+      </c>
+      <c r="D118" s="6">
+        <v>46110.709039351852</v>
+      </c>
+      <c r="E118" s="6">
+        <v>46110.811122685183</v>
+      </c>
+      <c r="F118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>14</v>
+      </c>
+      <c r="C119" s="5">
+        <v>46111</v>
+      </c>
+      <c r="D119" s="6">
+        <v>46111.740983796299</v>
+      </c>
+      <c r="E119" s="6">
+        <v>46111.937511574077</v>
+      </c>
+      <c r="F119">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120">
+        <v>14</v>
+      </c>
+      <c r="C120" s="5">
+        <v>46112</v>
+      </c>
+      <c r="D120" s="6">
+        <v>46112.729178240741</v>
+      </c>
+      <c r="E120" s="6">
+        <v>46112.920844907407</v>
+      </c>
+      <c r="F120">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2866,15 +3248,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46282368-3B73-4126-9CAF-0F4DBCD18058}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2891,7 +3273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2908,7 +3290,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2925,7 +3307,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2942,7 +3324,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2959,7 +3341,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2976,7 +3358,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2993,7 +3375,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3010,7 +3392,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3027,7 +3409,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3044,7 +3426,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3061,7 +3443,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3075,7 +3457,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3089,7 +3471,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3103,7 +3485,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3128,9 +3510,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC08066E-E57F-4738-8F85-A08D22304096}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3138,7 +3520,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3146,7 +3528,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3154,7 +3536,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3162,7 +3544,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3170,7 +3552,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3186,13 +3568,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1832BBAE-382C-4D1D-B62A-7A869140B59D}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -3200,7 +3582,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3208,7 +3590,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3216,7 +3598,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3224,7 +3606,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3232,7 +3614,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3240,7 +3622,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3248,7 +3630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3256,7 +3638,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3264,7 +3646,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3272,7 +3654,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3280,7 +3662,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3288,7 +3670,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3296,7 +3678,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3304,7 +3686,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3312,7 +3694,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3320,7 +3702,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3328,7 +3710,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3336,7 +3718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3344,7 +3726,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3352,7 +3734,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3360,7 +3742,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3368,7 +3750,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3376,7 +3758,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3384,7 +3766,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3392,7 +3774,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3400,7 +3782,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3408,7 +3790,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3416,7 +3798,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3432,9 +3814,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8190EB1-512E-4DA4-9E52-5BE9B6D9B4ED}">
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -3442,7 +3824,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2</v>
       </c>
@@ -3450,7 +3832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3458,7 +3840,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -3466,7 +3848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -3474,7 +3856,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
@@ -3482,7 +3864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>3</v>
       </c>
@@ -3490,7 +3872,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
@@ -3498,7 +3880,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>4</v>
       </c>
@@ -3506,7 +3888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>4</v>
       </c>
@@ -3514,7 +3896,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>6</v>
       </c>
@@ -3522,7 +3904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>6</v>
       </c>
@@ -3530,7 +3912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>7</v>
       </c>
@@ -3538,7 +3920,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>7</v>
       </c>
@@ -3546,7 +3928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>8</v>
       </c>
@@ -3554,7 +3936,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>8</v>
       </c>
@@ -3562,7 +3944,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>9</v>
       </c>
@@ -3570,7 +3952,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>9</v>
       </c>
@@ -3578,7 +3960,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>10</v>
       </c>
@@ -3586,7 +3968,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>10</v>
       </c>
@@ -3594,7 +3976,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>11</v>
       </c>
@@ -3602,7 +3984,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>11</v>
       </c>
@@ -3610,7 +3992,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>12</v>
       </c>
@@ -3618,7 +4000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>12</v>
       </c>
@@ -3626,7 +4008,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>13</v>
       </c>
@@ -3634,7 +4016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>13</v>
       </c>
@@ -3642,7 +4024,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>14</v>
       </c>
@@ -3650,7 +4032,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>14</v>
       </c>
@@ -3666,13 +4048,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B10FE8-D90F-4F6D-86B5-00602E8D2AAC}">
   <dimension ref="A1:B52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -3680,7 +4062,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3688,7 +4070,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3696,7 +4078,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3704,7 +4086,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3712,7 +4094,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3720,7 +4102,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3728,7 +4110,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3736,7 +4118,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3744,7 +4126,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3752,7 +4134,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3760,7 +4142,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3768,7 +4150,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3776,7 +4158,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3784,7 +4166,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3792,7 +4174,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3800,7 +4182,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3808,7 +4190,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3816,7 +4198,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3824,7 +4206,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3832,7 +4214,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3840,7 +4222,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3848,7 +4230,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3856,7 +4238,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3864,7 +4246,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3872,7 +4254,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3880,7 +4262,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3888,7 +4270,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3896,7 +4278,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3904,7 +4286,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3912,7 +4294,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3920,7 +4302,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3928,7 +4310,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3936,7 +4318,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3944,7 +4326,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3952,7 +4334,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3960,7 +4342,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3968,7 +4350,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3976,7 +4358,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3984,7 +4366,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3992,7 +4374,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4000,7 +4382,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4008,7 +4390,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4016,7 +4398,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4024,7 +4406,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4032,7 +4414,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4040,7 +4422,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4048,7 +4430,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4056,7 +4438,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4064,7 +4446,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4072,7 +4454,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4080,7 +4462,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4096,9 +4478,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95EFE99A-A4A1-483D-95A3-0523528D2F12}">
   <dimension ref="A1:B79"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -4106,7 +4488,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>4</v>
       </c>
@@ -4114,7 +4496,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>4</v>
       </c>
@@ -4122,7 +4504,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>4</v>
       </c>
@@ -4130,7 +4512,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4138,7 +4520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4146,7 +4528,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>4</v>
       </c>
@@ -4154,7 +4536,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4162,7 +4544,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4170,7 +4552,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4178,7 +4560,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4186,7 +4568,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4194,7 +4576,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2</v>
       </c>
@@ -4202,7 +4584,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2</v>
       </c>
@@ -4210,7 +4592,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2</v>
       </c>
@@ -4218,7 +4600,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2</v>
       </c>
@@ -4226,7 +4608,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2</v>
       </c>
@@ -4234,7 +4616,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2</v>
       </c>
@@ -4242,7 +4624,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>3</v>
       </c>
@@ -4250,7 +4632,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>3</v>
       </c>
@@ -4258,7 +4640,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>3</v>
       </c>
@@ -4266,7 +4648,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>3</v>
       </c>
@@ -4274,7 +4656,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>5</v>
       </c>
@@ -4282,7 +4664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>5</v>
       </c>
@@ -4290,7 +4672,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>5</v>
       </c>
@@ -4298,7 +4680,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>5</v>
       </c>
@@ -4306,7 +4688,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>6</v>
       </c>
@@ -4314,7 +4696,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>6</v>
       </c>
@@ -4322,7 +4704,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>6</v>
       </c>
@@ -4330,7 +4712,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>6</v>
       </c>
@@ -4338,7 +4720,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>6</v>
       </c>
@@ -4346,7 +4728,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>6</v>
       </c>
@@ -4354,7 +4736,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>7</v>
       </c>
@@ -4362,7 +4744,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>7</v>
       </c>
@@ -4370,7 +4752,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>7</v>
       </c>
@@ -4378,7 +4760,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>7</v>
       </c>
@@ -4386,7 +4768,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>7</v>
       </c>
@@ -4394,7 +4776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>7</v>
       </c>
@@ -4402,7 +4784,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>8</v>
       </c>
@@ -4410,7 +4792,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>8</v>
       </c>
@@ -4418,7 +4800,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>8</v>
       </c>
@@ -4426,7 +4808,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>8</v>
       </c>
@@ -4434,7 +4816,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>9</v>
       </c>
@@ -4442,7 +4824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>9</v>
       </c>
@@ -4450,7 +4832,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>9</v>
       </c>
@@ -4458,7 +4840,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>9</v>
       </c>
@@ -4466,7 +4848,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>9</v>
       </c>
@@ -4474,7 +4856,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>9</v>
       </c>
@@ -4482,7 +4864,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>9</v>
       </c>
@@ -4490,7 +4872,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>10</v>
       </c>
@@ -4498,7 +4880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>10</v>
       </c>
@@ -4506,7 +4888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>10</v>
       </c>
@@ -4514,7 +4896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>10</v>
       </c>
@@ -4522,7 +4904,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>10</v>
       </c>
@@ -4530,7 +4912,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>10</v>
       </c>
@@ -4538,7 +4920,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>11</v>
       </c>
@@ -4546,7 +4928,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>11</v>
       </c>
@@ -4554,7 +4936,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>11</v>
       </c>
@@ -4562,7 +4944,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>11</v>
       </c>
@@ -4570,7 +4952,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>11</v>
       </c>
@@ -4578,7 +4960,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>11</v>
       </c>
@@ -4586,7 +4968,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>12</v>
       </c>
@@ -4594,7 +4976,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>12</v>
       </c>
@@ -4602,7 +4984,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>12</v>
       </c>
@@ -4610,7 +4992,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>12</v>
       </c>
@@ -4618,7 +5000,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>12</v>
       </c>
@@ -4626,7 +5008,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>12</v>
       </c>
@@ -4634,7 +5016,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>13</v>
       </c>
@@ -4642,7 +5024,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>13</v>
       </c>
@@ -4650,7 +5032,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>13</v>
       </c>
@@ -4658,7 +5040,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>13</v>
       </c>
@@ -4666,7 +5048,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>13</v>
       </c>
@@ -4674,7 +5056,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>13</v>
       </c>
@@ -4682,7 +5064,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>14</v>
       </c>
@@ -4690,7 +5072,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>14</v>
       </c>
@@ -4698,7 +5080,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>14</v>
       </c>
@@ -4706,7 +5088,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>14</v>
       </c>
@@ -4714,7 +5096,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>14</v>
       </c>
@@ -4722,7 +5104,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Games added Replace Absolum No Nine Sols Shapez 2 Librarian
</commit_message>
<xml_diff>
--- a/New_Game_Time.xlsx
+++ b/New_Game_Time.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DAVIMUNO\Desktop\GitHub\Game_times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37425EDD-2FC8-4FEA-B0EE-D302091C188E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E41135A-3464-4A89-AB88-C28EE60FC507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sessions" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="166">
   <si>
     <t>SessionID</t>
   </si>
@@ -237,9 +237,6 @@
     <t>Roguelike Elements</t>
   </si>
   <si>
-    <t>Roguelite Elements</t>
-  </si>
-  <si>
     <t>Narrative-Driven</t>
   </si>
   <si>
@@ -490,6 +487,48 @@
   </si>
   <si>
     <t>Extraction Gameplay</t>
+  </si>
+  <si>
+    <t>Replaced</t>
+  </si>
+  <si>
+    <t>Shapez 2</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>Factory Building</t>
+  </si>
+  <si>
+    <t>Optimization-Focused</t>
+  </si>
+  <si>
+    <t>No Nine Sols</t>
+  </si>
+  <si>
+    <t>Absolum</t>
+  </si>
+  <si>
+    <t>Librarian: Tidy Up the Arcane Library</t>
+  </si>
+  <si>
+    <t>Sad Cat Studios</t>
+  </si>
+  <si>
+    <t>Thunderful Publishing</t>
+  </si>
+  <si>
+    <t>Red Candle Games</t>
+  </si>
+  <si>
+    <t>Guard Crush Games</t>
+  </si>
+  <si>
+    <t>ArtRising</t>
+  </si>
+  <si>
+    <t>Tobspr Games</t>
   </si>
 </sst>
 </file>
@@ -553,7 +592,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -830,17 +877,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F138"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" customWidth="1"/>
-    <col min="5" max="5" width="16.7265625" customWidth="1"/>
-    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -860,7 +907,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -880,7 +927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -900,7 +947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -920,7 +967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -940,7 +987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -960,7 +1007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -980,7 +1027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1000,7 +1047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1020,7 +1067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1040,7 +1087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1060,7 +1107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1080,7 +1127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1100,7 +1147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1120,7 +1167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1140,7 +1187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1160,7 +1207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1180,7 +1227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1200,7 +1247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1220,7 +1267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1240,7 +1287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1260,7 +1307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1280,7 +1327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1300,7 +1347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1320,7 +1367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1340,7 +1387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1360,7 +1407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1380,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1400,7 +1447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1420,7 +1467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1440,7 +1487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1460,7 +1507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1480,7 +1527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1500,7 +1547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1520,7 +1567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1540,7 +1587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1560,7 +1607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1580,7 +1627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1600,7 +1647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1620,7 +1667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1640,7 +1687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1660,7 +1707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1680,7 +1727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1700,7 +1747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1720,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1740,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1760,7 +1807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1780,7 +1827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1800,7 +1847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1820,7 +1867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1840,7 +1887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1860,7 +1907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1880,7 +1927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1900,7 +1947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1920,7 +1967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1940,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1960,7 +2007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1980,7 +2027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2000,7 +2047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2020,7 +2067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2040,7 +2087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2060,7 +2107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2080,7 +2127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2100,7 +2147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2120,7 +2167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2140,7 +2187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2160,7 +2207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2180,7 +2227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2200,7 +2247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2220,7 +2267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2240,7 +2287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2260,7 +2307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2280,7 +2327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2300,7 +2347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2320,7 +2367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2340,7 +2387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2360,7 +2407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2380,7 +2427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2400,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2420,7 +2467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2440,7 +2487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2460,7 +2507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2480,7 +2527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2500,7 +2547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2520,7 +2567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2540,7 +2587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2560,7 +2607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2580,7 +2627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2600,7 +2647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2620,7 +2667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2640,7 +2687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2660,7 +2707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2680,7 +2727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2700,7 +2747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2720,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2740,7 +2787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2760,7 +2807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2780,7 +2827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2791,16 +2838,16 @@
         <v>46101</v>
       </c>
       <c r="D98" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E98" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="E98" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="F98" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2811,16 +2858,16 @@
         <v>46101</v>
       </c>
       <c r="D99" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E99" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E99" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="F99" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2831,16 +2878,16 @@
         <v>46101</v>
       </c>
       <c r="D100" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E100" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E100" s="4" t="s">
-        <v>130</v>
-      </c>
       <c r="F100" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2851,16 +2898,16 @@
         <v>46101</v>
       </c>
       <c r="D101" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E101" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E101" s="4" t="s">
-        <v>132</v>
-      </c>
       <c r="F101" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -2880,7 +2927,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -2900,7 +2947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -2920,7 +2967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -2940,7 +2987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -2960,7 +3007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -2980,7 +3027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3000,7 +3047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3020,7 +3067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3040,7 +3087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3060,7 +3107,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3080,7 +3127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3100,7 +3147,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3120,7 +3167,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3140,7 +3187,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3160,7 +3207,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3180,7 +3227,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3200,7 +3247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -3220,7 +3267,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -3240,7 +3287,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -3260,7 +3307,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3280,7 +3327,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3300,7 +3347,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3320,7 +3367,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3340,7 +3387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3360,7 +3407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3380,7 +3427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3400,7 +3447,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3420,7 +3467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3440,7 +3487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3460,7 +3507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -3480,7 +3527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -3500,7 +3547,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -3520,7 +3567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -3540,7 +3587,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -3560,7 +3607,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -3580,7 +3627,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -3607,16 +3654,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46282368-3B73-4126-9CAF-0F4DBCD18058}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -3633,233 +3680,303 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
         <v>84</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" t="s">
         <v>85</v>
       </c>
-      <c r="D2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
         <v>88</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" t="s">
         <v>92</v>
       </c>
-      <c r="E4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" t="s">
         <v>96</v>
       </c>
-      <c r="E5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" t="s">
         <v>100</v>
       </c>
-      <c r="E6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s">
         <v>107</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" t="s">
         <v>118</v>
       </c>
-      <c r="E10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" t="s">
         <v>122</v>
       </c>
-      <c r="E11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="E15" t="s">
-        <v>143</v>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3870,9 +3987,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC08066E-E57F-4738-8F85-A08D22304096}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3880,7 +3997,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3888,7 +4005,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3896,7 +4013,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3904,7 +4021,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3912,7 +4029,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3928,13 +4045,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1832BBAE-382C-4D1D-B62A-7A869140B59D}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -3942,7 +4059,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3950,7 +4067,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3958,7 +4075,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3966,7 +4083,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3974,7 +4091,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3982,7 +4099,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3990,7 +4107,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3998,7 +4115,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4006,7 +4123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4014,7 +4131,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4022,7 +4139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4030,7 +4147,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4038,7 +4155,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4046,7 +4163,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4054,7 +4171,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4062,7 +4179,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4070,7 +4187,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -4078,7 +4195,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4086,7 +4203,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4094,7 +4211,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4102,7 +4219,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4110,7 +4227,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4118,7 +4235,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4126,7 +4243,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4134,7 +4251,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4142,7 +4259,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4150,7 +4267,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4158,12 +4275,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -4173,10 +4290,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8190EB1-512E-4DA4-9E52-5BE9B6D9B4ED}">
-  <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -4184,7 +4301,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -4192,7 +4309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4200,7 +4317,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -4208,7 +4325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -4216,7 +4333,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -4224,7 +4341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -4232,7 +4349,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -4240,7 +4357,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4</v>
       </c>
@@ -4248,7 +4365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -4256,7 +4373,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>6</v>
       </c>
@@ -4264,7 +4381,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -4272,7 +4389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
@@ -4280,7 +4397,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7</v>
       </c>
@@ -4288,7 +4405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>8</v>
       </c>
@@ -4296,7 +4413,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>8</v>
       </c>
@@ -4304,7 +4421,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>9</v>
       </c>
@@ -4312,7 +4429,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9</v>
       </c>
@@ -4320,7 +4437,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>10</v>
       </c>
@@ -4328,7 +4445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>10</v>
       </c>
@@ -4336,7 +4453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>11</v>
       </c>
@@ -4344,7 +4461,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>11</v>
       </c>
@@ -4352,7 +4469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>12</v>
       </c>
@@ -4360,7 +4477,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>12</v>
       </c>
@@ -4368,7 +4485,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>13</v>
       </c>
@@ -4376,7 +4493,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>13</v>
       </c>
@@ -4384,7 +4501,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>14</v>
       </c>
@@ -4392,12 +4509,92 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>14</v>
       </c>
       <c r="B28">
         <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>15</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>15</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>16</v>
+      </c>
+      <c r="B31">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>16</v>
+      </c>
+      <c r="B32">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>17</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>17</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>18</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>18</v>
+      </c>
+      <c r="B36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>19</v>
+      </c>
+      <c r="B37">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>19</v>
+      </c>
+      <c r="B38">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -4407,14 +4604,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B10FE8-D90F-4F6D-86B5-00602E8D2AAC}">
-  <dimension ref="A1:B52"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -4422,7 +4619,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4430,7 +4627,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4438,7 +4635,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4446,7 +4643,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4454,7 +4651,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4462,7 +4659,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4470,7 +4667,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4478,7 +4675,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4486,7 +4683,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4494,7 +4691,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4502,7 +4699,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4510,7 +4707,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4518,7 +4715,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4526,7 +4723,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4534,7 +4731,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4542,7 +4739,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4550,7 +4747,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -4558,7 +4755,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4566,7 +4763,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4574,7 +4771,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4582,252 +4779,268 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -4837,10 +5050,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95EFE99A-A4A1-483D-95A3-0523528D2F12}">
-  <dimension ref="A1:B79"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B103"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -4848,7 +5061,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>4</v>
       </c>
@@ -4856,7 +5069,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>4</v>
       </c>
@@ -4864,7 +5077,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -4872,7 +5085,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4880,7 +5093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4888,7 +5101,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -4896,7 +5109,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4904,7 +5117,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4912,7 +5125,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4920,7 +5133,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4928,7 +5141,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4936,7 +5149,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -4944,7 +5157,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -4952,7 +5165,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -4960,7 +5173,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -4968,7 +5181,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -4976,7 +5189,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -4984,7 +5197,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -4992,7 +5205,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -5000,7 +5213,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -5008,7 +5221,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -5016,7 +5229,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>5</v>
       </c>
@@ -5024,7 +5237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>5</v>
       </c>
@@ -5032,7 +5245,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>5</v>
       </c>
@@ -5040,7 +5253,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>5</v>
       </c>
@@ -5048,7 +5261,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>6</v>
       </c>
@@ -5056,7 +5269,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>6</v>
       </c>
@@ -5064,7 +5277,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>6</v>
       </c>
@@ -5072,7 +5285,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>6</v>
       </c>
@@ -5080,7 +5293,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>6</v>
       </c>
@@ -5088,7 +5301,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>6</v>
       </c>
@@ -5096,7 +5309,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>7</v>
       </c>
@@ -5104,7 +5317,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>7</v>
       </c>
@@ -5112,7 +5325,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>7</v>
       </c>
@@ -5120,7 +5333,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>7</v>
       </c>
@@ -5128,7 +5341,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>7</v>
       </c>
@@ -5136,7 +5349,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>7</v>
       </c>
@@ -5144,7 +5357,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>8</v>
       </c>
@@ -5152,7 +5365,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>8</v>
       </c>
@@ -5160,7 +5373,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>8</v>
       </c>
@@ -5168,7 +5381,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>8</v>
       </c>
@@ -5176,7 +5389,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>9</v>
       </c>
@@ -5184,7 +5397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>9</v>
       </c>
@@ -5192,7 +5405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>9</v>
       </c>
@@ -5200,7 +5413,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -5208,7 +5421,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>9</v>
       </c>
@@ -5216,7 +5429,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>9</v>
       </c>
@@ -5224,7 +5437,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>9</v>
       </c>
@@ -5232,7 +5445,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>10</v>
       </c>
@@ -5240,7 +5453,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>10</v>
       </c>
@@ -5248,7 +5461,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10</v>
       </c>
@@ -5256,7 +5469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10</v>
       </c>
@@ -5264,7 +5477,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10</v>
       </c>
@@ -5272,7 +5485,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10</v>
       </c>
@@ -5280,7 +5493,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>11</v>
       </c>
@@ -5288,7 +5501,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>11</v>
       </c>
@@ -5296,15 +5509,15 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>11</v>
       </c>
       <c r="B58">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>11</v>
       </c>
@@ -5312,7 +5525,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>11</v>
       </c>
@@ -5320,7 +5533,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>11</v>
       </c>
@@ -5328,7 +5541,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>12</v>
       </c>
@@ -5336,7 +5549,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>12</v>
       </c>
@@ -5344,7 +5557,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>12</v>
       </c>
@@ -5352,7 +5565,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>12</v>
       </c>
@@ -5360,7 +5573,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>12</v>
       </c>
@@ -5368,7 +5581,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>12</v>
       </c>
@@ -5376,7 +5589,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>13</v>
       </c>
@@ -5384,7 +5597,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>13</v>
       </c>
@@ -5392,7 +5605,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>13</v>
       </c>
@@ -5400,7 +5613,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>13</v>
       </c>
@@ -5408,7 +5621,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>13</v>
       </c>
@@ -5416,7 +5629,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>13</v>
       </c>
@@ -5424,7 +5637,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>14</v>
       </c>
@@ -5432,7 +5645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>14</v>
       </c>
@@ -5440,7 +5653,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>14</v>
       </c>
@@ -5448,7 +5661,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>14</v>
       </c>
@@ -5456,7 +5669,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>14</v>
       </c>
@@ -5464,12 +5677,204 @@
         <v>28</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>14</v>
       </c>
       <c r="B79">
         <v>14</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>15</v>
+      </c>
+      <c r="B80">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>15</v>
+      </c>
+      <c r="B81">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>15</v>
+      </c>
+      <c r="B82">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>15</v>
+      </c>
+      <c r="B83">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>15</v>
+      </c>
+      <c r="B84">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>15</v>
+      </c>
+      <c r="B85">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>16</v>
+      </c>
+      <c r="B86">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>16</v>
+      </c>
+      <c r="B87">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>16</v>
+      </c>
+      <c r="B88">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>16</v>
+      </c>
+      <c r="B89">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>16</v>
+      </c>
+      <c r="B90">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>17</v>
+      </c>
+      <c r="B91">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>17</v>
+      </c>
+      <c r="B92">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>17</v>
+      </c>
+      <c r="B93">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>17</v>
+      </c>
+      <c r="B94">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>17</v>
+      </c>
+      <c r="B95">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>18</v>
+      </c>
+      <c r="B96">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>18</v>
+      </c>
+      <c r="B97">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>18</v>
+      </c>
+      <c r="B98">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>18</v>
+      </c>
+      <c r="B99">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>18</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>19</v>
+      </c>
+      <c r="B101">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>19</v>
+      </c>
+      <c r="B102">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>19</v>
+      </c>
+      <c r="B103">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add sesion from 138 - 198
</commit_message>
<xml_diff>
--- a/New_Game_Time.xlsx
+++ b/New_Game_Time.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DAVIMUNO\Desktop\GitHub\Game_times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E41135A-3464-4A89-AB88-C28EE60FC507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72028AF3-BF24-4A71-868A-A209F6D1C284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -592,15 +592,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -876,12 +868,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -3645,6 +3637,1226 @@
       </c>
       <c r="F138" s="2">
         <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139">
+        <v>14</v>
+      </c>
+      <c r="C139" s="3">
+        <v>46125</v>
+      </c>
+      <c r="D139" s="4">
+        <v>46125.75277777778</v>
+      </c>
+      <c r="E139" s="4">
+        <v>46125.92291666667</v>
+      </c>
+      <c r="F139" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140">
+        <v>15</v>
+      </c>
+      <c r="C140" s="3">
+        <v>46126</v>
+      </c>
+      <c r="D140" s="4">
+        <v>46126.731944444444</v>
+      </c>
+      <c r="E140" s="4">
+        <v>46126.820138888892</v>
+      </c>
+      <c r="F140" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141">
+        <v>15</v>
+      </c>
+      <c r="C141" s="3">
+        <v>46127</v>
+      </c>
+      <c r="D141" s="4">
+        <v>46127.788888888892</v>
+      </c>
+      <c r="E141" s="4">
+        <v>46127.833333333336</v>
+      </c>
+      <c r="F141" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142">
+        <v>15</v>
+      </c>
+      <c r="C142" s="3">
+        <v>46127</v>
+      </c>
+      <c r="D142" s="4">
+        <v>46127.847916666666</v>
+      </c>
+      <c r="E142" s="4">
+        <v>46127.916666666664</v>
+      </c>
+      <c r="F142" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143">
+        <v>14</v>
+      </c>
+      <c r="C143" s="3">
+        <v>46128</v>
+      </c>
+      <c r="D143" s="4">
+        <v>46128.28125</v>
+      </c>
+      <c r="E143" s="4">
+        <v>46128.322916666664</v>
+      </c>
+      <c r="F143" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144">
+        <v>14</v>
+      </c>
+      <c r="C144" s="3">
+        <v>46128</v>
+      </c>
+      <c r="D144" s="4">
+        <v>46128.709027777775</v>
+      </c>
+      <c r="E144" s="4">
+        <v>46128.830555555556</v>
+      </c>
+      <c r="F144" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145">
+        <v>14</v>
+      </c>
+      <c r="C145" s="3">
+        <v>46130</v>
+      </c>
+      <c r="D145" s="4">
+        <v>46130.75</v>
+      </c>
+      <c r="E145" s="4">
+        <v>46130.876388888886</v>
+      </c>
+      <c r="F145" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146">
+        <v>14</v>
+      </c>
+      <c r="C146" s="3">
+        <v>46132</v>
+      </c>
+      <c r="D146" s="4">
+        <v>46132.743055555555</v>
+      </c>
+      <c r="E146" s="4">
+        <v>46132.833333333336</v>
+      </c>
+      <c r="F146" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147">
+        <v>14</v>
+      </c>
+      <c r="C147" s="3">
+        <v>46133</v>
+      </c>
+      <c r="D147" s="4">
+        <v>46133.732638888891</v>
+      </c>
+      <c r="E147" s="4">
+        <v>46133.847222222219</v>
+      </c>
+      <c r="F147" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148">
+        <v>18</v>
+      </c>
+      <c r="C148" s="3">
+        <v>46134</v>
+      </c>
+      <c r="D148" s="4">
+        <v>46134.75277777778</v>
+      </c>
+      <c r="E148" s="4">
+        <v>46134.902083333334</v>
+      </c>
+      <c r="F148" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149">
+        <v>18</v>
+      </c>
+      <c r="C149" s="3">
+        <v>46135</v>
+      </c>
+      <c r="D149" s="4">
+        <v>46135.307638888888</v>
+      </c>
+      <c r="E149" s="4">
+        <v>46135.34375</v>
+      </c>
+      <c r="F149" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150">
+        <v>18</v>
+      </c>
+      <c r="C150" s="3">
+        <v>46135</v>
+      </c>
+      <c r="D150" s="4">
+        <v>46135.55</v>
+      </c>
+      <c r="E150" s="4">
+        <v>46135.574305555558</v>
+      </c>
+      <c r="F150" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151">
+        <v>18</v>
+      </c>
+      <c r="C151" s="3">
+        <v>46135</v>
+      </c>
+      <c r="D151" s="4">
+        <v>46135.715277777781</v>
+      </c>
+      <c r="E151" s="4">
+        <v>46135.90625</v>
+      </c>
+      <c r="F151" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152">
+        <v>16</v>
+      </c>
+      <c r="C152" s="3">
+        <v>46136</v>
+      </c>
+      <c r="D152" s="4">
+        <v>46136.893750000003</v>
+      </c>
+      <c r="E152" s="4">
+        <v>46136.999305555553</v>
+      </c>
+      <c r="F152" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153">
+        <v>16</v>
+      </c>
+      <c r="C153" s="3">
+        <v>46137</v>
+      </c>
+      <c r="D153" s="4">
+        <v>46137</v>
+      </c>
+      <c r="E153" s="4">
+        <v>46137.069444444445</v>
+      </c>
+      <c r="F153" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154">
+        <v>16</v>
+      </c>
+      <c r="C154" s="3">
+        <v>46137</v>
+      </c>
+      <c r="D154" s="4">
+        <v>46137.4375</v>
+      </c>
+      <c r="E154" s="4">
+        <v>46137.765277777777</v>
+      </c>
+      <c r="F154" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155">
+        <v>18</v>
+      </c>
+      <c r="C155" s="3">
+        <v>46137</v>
+      </c>
+      <c r="D155" s="4">
+        <v>46137.811111111114</v>
+      </c>
+      <c r="E155" s="4">
+        <v>46137.90625</v>
+      </c>
+      <c r="F155" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156">
+        <v>14</v>
+      </c>
+      <c r="C156" s="3">
+        <v>46137</v>
+      </c>
+      <c r="D156" s="4">
+        <v>46137.92291666667</v>
+      </c>
+      <c r="E156" s="4">
+        <v>46138.06527777778</v>
+      </c>
+      <c r="F156" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157">
+        <v>14</v>
+      </c>
+      <c r="C157" s="3">
+        <v>46138</v>
+      </c>
+      <c r="D157" s="4">
+        <v>46138.581250000003</v>
+      </c>
+      <c r="E157" s="4">
+        <v>46138.630555555559</v>
+      </c>
+      <c r="F157" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158">
+        <v>16</v>
+      </c>
+      <c r="C158" s="3">
+        <v>46138</v>
+      </c>
+      <c r="D158" s="4">
+        <v>46138.78125</v>
+      </c>
+      <c r="E158" s="4">
+        <v>46138.999305555553</v>
+      </c>
+      <c r="F158" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159">
+        <v>16</v>
+      </c>
+      <c r="C159" s="3">
+        <v>46139</v>
+      </c>
+      <c r="D159" s="4">
+        <v>46139</v>
+      </c>
+      <c r="E159" s="4">
+        <v>46139.021527777775</v>
+      </c>
+      <c r="F159" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160">
+        <v>16</v>
+      </c>
+      <c r="C160" s="3">
+        <v>46139</v>
+      </c>
+      <c r="D160" s="4">
+        <v>46139.688194444447</v>
+      </c>
+      <c r="E160" s="4">
+        <v>46139.999305555553</v>
+      </c>
+      <c r="F160" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161">
+        <v>16</v>
+      </c>
+      <c r="C161" s="3">
+        <v>46140</v>
+      </c>
+      <c r="D161" s="4">
+        <v>46140.780555555553</v>
+      </c>
+      <c r="E161" s="4">
+        <v>46140.999305555553</v>
+      </c>
+      <c r="F161" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162">
+        <v>16</v>
+      </c>
+      <c r="C162" s="3">
+        <v>46141</v>
+      </c>
+      <c r="D162" s="4">
+        <v>46141</v>
+      </c>
+      <c r="E162" s="4">
+        <v>46141.008333333331</v>
+      </c>
+      <c r="F162" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163">
+        <v>16</v>
+      </c>
+      <c r="C163" s="3">
+        <v>46144</v>
+      </c>
+      <c r="D163" s="4">
+        <v>46144.895833333336</v>
+      </c>
+      <c r="E163" s="4">
+        <v>46144.999305555553</v>
+      </c>
+      <c r="F163" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164">
+        <v>16</v>
+      </c>
+      <c r="C164" s="3">
+        <v>46145</v>
+      </c>
+      <c r="D164" s="4">
+        <v>46145</v>
+      </c>
+      <c r="E164" s="4">
+        <v>46145.105555555558</v>
+      </c>
+      <c r="F164" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165">
+        <v>16</v>
+      </c>
+      <c r="C165" s="3">
+        <v>46145</v>
+      </c>
+      <c r="D165" s="4">
+        <v>46145.388888888891</v>
+      </c>
+      <c r="E165" s="4">
+        <v>46145.413888888892</v>
+      </c>
+      <c r="F165" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166">
+        <v>14</v>
+      </c>
+      <c r="C166" s="3">
+        <v>46145</v>
+      </c>
+      <c r="D166" s="4">
+        <v>46145.869444444441</v>
+      </c>
+      <c r="E166" s="4">
+        <v>46145.915277777778</v>
+      </c>
+      <c r="F166" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167">
+        <v>14</v>
+      </c>
+      <c r="C167" s="3">
+        <v>46146</v>
+      </c>
+      <c r="D167" s="4">
+        <v>46146.832638888889</v>
+      </c>
+      <c r="E167" s="4">
+        <v>46146.85833333333</v>
+      </c>
+      <c r="F167" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168">
+        <v>14</v>
+      </c>
+      <c r="C168" s="3">
+        <v>46148</v>
+      </c>
+      <c r="D168" s="4">
+        <v>46148.919444444444</v>
+      </c>
+      <c r="E168" s="4">
+        <v>46148.999305555553</v>
+      </c>
+      <c r="F168" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169">
+        <v>14</v>
+      </c>
+      <c r="C169" s="3">
+        <v>46149</v>
+      </c>
+      <c r="D169" s="4">
+        <v>46149</v>
+      </c>
+      <c r="E169" s="4">
+        <v>46149.024305555555</v>
+      </c>
+      <c r="F169" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170">
+        <v>18</v>
+      </c>
+      <c r="C170" s="3">
+        <v>46149</v>
+      </c>
+      <c r="D170" s="4">
+        <v>46149.795138888891</v>
+      </c>
+      <c r="E170" s="4">
+        <v>46149.960416666669</v>
+      </c>
+      <c r="F170" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171">
+        <v>14</v>
+      </c>
+      <c r="C171" s="3">
+        <v>46150</v>
+      </c>
+      <c r="D171" s="4">
+        <v>46150.591666666667</v>
+      </c>
+      <c r="E171" s="4">
+        <v>46150.634027777778</v>
+      </c>
+      <c r="F171" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172">
+        <v>14</v>
+      </c>
+      <c r="C172" s="3">
+        <v>46150</v>
+      </c>
+      <c r="D172" s="4">
+        <v>46150.895833333336</v>
+      </c>
+      <c r="E172" s="4">
+        <v>46150.958333333336</v>
+      </c>
+      <c r="F172" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173">
+        <v>14</v>
+      </c>
+      <c r="C173" s="3">
+        <v>46151</v>
+      </c>
+      <c r="D173" s="4">
+        <v>46151.803472222222</v>
+      </c>
+      <c r="E173" s="4">
+        <v>46151.999305555553</v>
+      </c>
+      <c r="F173" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174">
+        <v>14</v>
+      </c>
+      <c r="C174" s="3">
+        <v>46152</v>
+      </c>
+      <c r="D174" s="4">
+        <v>46152</v>
+      </c>
+      <c r="E174" s="4">
+        <v>46152.083333333336</v>
+      </c>
+      <c r="F174" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175">
+        <v>14</v>
+      </c>
+      <c r="C175" s="3">
+        <v>46152</v>
+      </c>
+      <c r="D175" s="4">
+        <v>46152.36041666667</v>
+      </c>
+      <c r="E175" s="4">
+        <v>46152.395138888889</v>
+      </c>
+      <c r="F175" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176">
+        <v>14</v>
+      </c>
+      <c r="C176" s="3">
+        <v>46152</v>
+      </c>
+      <c r="D176" s="4">
+        <v>46152.632638888892</v>
+      </c>
+      <c r="E176" s="4">
+        <v>46152.732638888891</v>
+      </c>
+      <c r="F176" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177">
+        <v>17</v>
+      </c>
+      <c r="C177" s="3">
+        <v>46153</v>
+      </c>
+      <c r="D177" s="4">
+        <v>46153.759722222225</v>
+      </c>
+      <c r="E177" s="4">
+        <v>46153.786805555559</v>
+      </c>
+      <c r="F177" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178">
+        <v>17</v>
+      </c>
+      <c r="C178" s="3">
+        <v>46153</v>
+      </c>
+      <c r="D178" s="4">
+        <v>46153.838194444441</v>
+      </c>
+      <c r="E178" s="4">
+        <v>46153.881944444445</v>
+      </c>
+      <c r="F178" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179">
+        <v>14</v>
+      </c>
+      <c r="C179" s="3">
+        <v>46154</v>
+      </c>
+      <c r="D179" s="4">
+        <v>46154.768750000003</v>
+      </c>
+      <c r="E179" s="4">
+        <v>46154.833333333336</v>
+      </c>
+      <c r="F179" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180">
+        <v>17</v>
+      </c>
+      <c r="C180" s="3">
+        <v>46154</v>
+      </c>
+      <c r="D180" s="4">
+        <v>46154.852083333331</v>
+      </c>
+      <c r="E180" s="4">
+        <v>46154.881944444445</v>
+      </c>
+      <c r="F180" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181">
+        <v>14</v>
+      </c>
+      <c r="C181" s="3">
+        <v>46157</v>
+      </c>
+      <c r="D181" s="4">
+        <v>46157.510416666664</v>
+      </c>
+      <c r="E181" s="4">
+        <v>46157.565972222219</v>
+      </c>
+      <c r="F181" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182">
+        <v>14</v>
+      </c>
+      <c r="C182" s="3">
+        <v>46157</v>
+      </c>
+      <c r="D182" s="4">
+        <v>46157.656944444447</v>
+      </c>
+      <c r="E182" s="4">
+        <v>46157.734027777777</v>
+      </c>
+      <c r="F182" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183">
+        <v>19</v>
+      </c>
+      <c r="C183" s="3">
+        <v>46157</v>
+      </c>
+      <c r="D183" s="4">
+        <v>46157.762499999997</v>
+      </c>
+      <c r="E183" s="4">
+        <v>46157.886111111111</v>
+      </c>
+      <c r="F183" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184">
+        <v>19</v>
+      </c>
+      <c r="C184" s="3">
+        <v>46157</v>
+      </c>
+      <c r="D184" s="4">
+        <v>46157.905555555553</v>
+      </c>
+      <c r="E184" s="4">
+        <v>46157.999305555553</v>
+      </c>
+      <c r="F184" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185">
+        <v>19</v>
+      </c>
+      <c r="C185" s="3">
+        <v>46158</v>
+      </c>
+      <c r="D185" s="4">
+        <v>46158</v>
+      </c>
+      <c r="E185" s="4">
+        <v>46158.102777777778</v>
+      </c>
+      <c r="F185" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186">
+        <v>14</v>
+      </c>
+      <c r="C186" s="3">
+        <v>46158</v>
+      </c>
+      <c r="D186" s="4">
+        <v>46158.564583333333</v>
+      </c>
+      <c r="E186" s="4">
+        <v>46158.582638888889</v>
+      </c>
+      <c r="F186" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187">
+        <v>14</v>
+      </c>
+      <c r="C187" s="3">
+        <v>46158</v>
+      </c>
+      <c r="D187" s="4">
+        <v>46158.591666666667</v>
+      </c>
+      <c r="E187" s="4">
+        <v>46158.690972222219</v>
+      </c>
+      <c r="F187" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188">
+        <v>17</v>
+      </c>
+      <c r="C188" s="3">
+        <v>46158</v>
+      </c>
+      <c r="D188" s="4">
+        <v>46158.976388888892</v>
+      </c>
+      <c r="E188" s="4">
+        <v>46158.999305555553</v>
+      </c>
+      <c r="F188" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189">
+        <v>17</v>
+      </c>
+      <c r="C189" s="3">
+        <v>46159</v>
+      </c>
+      <c r="D189" s="4">
+        <v>46159</v>
+      </c>
+      <c r="E189" s="4">
+        <v>46159.020833333336</v>
+      </c>
+      <c r="F189" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190">
+        <v>16</v>
+      </c>
+      <c r="C190" s="3">
+        <v>46159</v>
+      </c>
+      <c r="D190" s="4">
+        <v>46159.47152777778</v>
+      </c>
+      <c r="E190" s="4">
+        <v>46159.552083333336</v>
+      </c>
+      <c r="F190" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191">
+        <v>16</v>
+      </c>
+      <c r="C191" s="3">
+        <v>46159</v>
+      </c>
+      <c r="D191" s="4">
+        <v>46159.823611111111</v>
+      </c>
+      <c r="E191" s="4">
+        <v>46159.884722222225</v>
+      </c>
+      <c r="F191" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192">
+        <v>16</v>
+      </c>
+      <c r="C192" s="3">
+        <v>46159</v>
+      </c>
+      <c r="D192" s="4">
+        <v>46159.93472222222</v>
+      </c>
+      <c r="E192" s="4">
+        <v>46159.999305555553</v>
+      </c>
+      <c r="F192" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193">
+        <v>16</v>
+      </c>
+      <c r="C193" s="3">
+        <v>46163</v>
+      </c>
+      <c r="D193" s="4">
+        <v>46163.926388888889</v>
+      </c>
+      <c r="E193" s="4">
+        <v>46163.999305555553</v>
+      </c>
+      <c r="F193" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194">
+        <v>16</v>
+      </c>
+      <c r="C194" s="3">
+        <v>46164</v>
+      </c>
+      <c r="D194" s="4">
+        <v>46164</v>
+      </c>
+      <c r="E194" s="4">
+        <v>46164.020833333336</v>
+      </c>
+      <c r="F194" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195">
+        <v>14</v>
+      </c>
+      <c r="C195" s="3">
+        <v>46164</v>
+      </c>
+      <c r="D195" s="4">
+        <v>46164.771527777775</v>
+      </c>
+      <c r="E195" s="4">
+        <v>46164.847222222219</v>
+      </c>
+      <c r="F195" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196">
+        <v>14</v>
+      </c>
+      <c r="C196" s="3">
+        <v>46165</v>
+      </c>
+      <c r="D196" s="4">
+        <v>46165.625</v>
+      </c>
+      <c r="E196" s="4">
+        <v>46165.863194444442</v>
+      </c>
+      <c r="F196" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197">
+        <v>16</v>
+      </c>
+      <c r="C197" s="3">
+        <v>46165</v>
+      </c>
+      <c r="D197" s="4">
+        <v>46165.902083333334</v>
+      </c>
+      <c r="E197" s="4">
+        <v>46165.999305555553</v>
+      </c>
+      <c r="F197" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198">
+        <v>16</v>
+      </c>
+      <c r="C198" s="3">
+        <v>46166</v>
+      </c>
+      <c r="D198" s="4">
+        <v>46166</v>
+      </c>
+      <c r="E198" s="4">
+        <v>46166.104166666664</v>
+      </c>
+      <c r="F198" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199">
+        <v>16</v>
+      </c>
+      <c r="C199" s="3">
+        <v>46166</v>
+      </c>
+      <c r="D199" s="4">
+        <v>46166.878472222219</v>
+      </c>
+      <c r="E199" s="4">
+        <v>46166.984722222223</v>
+      </c>
+      <c r="F199" s="2">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>